<commit_message>
Daily slate 2026-05-16 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-15.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-15.xlsx
@@ -471,13 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="G2" t="n">
+        <v>53.3</v>
       </c>
     </row>
     <row r="3">
@@ -497,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="4">
@@ -526,13 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>41.7</v>
       </c>
     </row>
     <row r="5">
@@ -552,13 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="G5" t="n">
+        <v>62.5</v>
       </c>
     </row>
     <row r="6">
@@ -578,13 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="G6" t="n">
+        <v>53.1</v>
       </c>
     </row>
     <row r="7">
@@ -604,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="8">
@@ -633,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>187</v>
+        <v>795</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>300</v>
       </c>
       <c r="F8" t="n">
-        <v>151</v>
+        <v>495</v>
       </c>
       <c r="G8" t="n">
-        <v>19.3</v>
+        <v>37.7</v>
       </c>
     </row>
     <row r="9">
@@ -662,13 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>158</v>
+      </c>
+      <c r="G9" t="n">
+        <v>50.9</v>
       </c>
     </row>
     <row r="10">
@@ -688,13 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>675</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>225</v>
+      </c>
+      <c r="G10" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="11">
@@ -714,13 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>492</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>318</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>174</v>
+      </c>
+      <c r="G11" t="n">
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -740,13 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>86</v>
+      </c>
+      <c r="G12" t="n">
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -766,13 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>103</v>
+      </c>
+      <c r="G13" t="n">
+        <v>56.7</v>
       </c>
     </row>
     <row r="14">
@@ -792,13 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>129</v>
+      </c>
+      <c r="G14" t="n">
+        <v>31.4</v>
       </c>
     </row>
     <row r="15">
@@ -818,13 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>242</v>
+      </c>
+      <c r="G15" t="n">
+        <v>22.4</v>
       </c>
     </row>
     <row r="16">
@@ -844,13 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>109</v>
+      </c>
+      <c r="G16" t="n">
+        <v>23.8</v>
       </c>
     </row>
     <row r="17">
@@ -870,13 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>2430</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>532</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1898</v>
+      </c>
+      <c r="G17" t="n">
+        <v>21.9</v>
       </c>
     </row>
   </sheetData>
@@ -1066,32 +1105,59 @@
           <t>Elite</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>80.40000000000001</v>
+      </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>56</v>
+      </c>
+      <c r="D2" t="n">
+        <v>67.3</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>55</v>
+      </c>
+      <c r="F2" t="n">
+        <v>64.59999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>48</v>
+      </c>
+      <c r="H2" t="n">
+        <v>62.4</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>85</v>
+      </c>
+      <c r="J2" t="n">
+        <v>50</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="L2" t="n">
+        <v>26.8</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>56</v>
+      </c>
+      <c r="N2" t="n">
+        <v>17.9</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="P2" t="n">
+        <v>28.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>56</v>
+      </c>
+      <c r="R2" t="n">
+        <v>50</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -1099,20 +1165,35 @@
       <c r="W2" t="n">
         <v>0</v>
       </c>
+      <c r="X2" t="n">
+        <v>47.6</v>
+      </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>206</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>84.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>63.2</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>28.6</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>62</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -1121,53 +1202,98 @@
           <t>Above Avg</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>72.40000000000001</v>
+      </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>174</v>
+      </c>
+      <c r="D3" t="n">
+        <v>63.4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>112</v>
+      </c>
+      <c r="F3" t="n">
+        <v>68.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>73</v>
+      </c>
+      <c r="H3" t="n">
+        <v>41.3</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>63</v>
+      </c>
+      <c r="J3" t="n">
+        <v>66.7</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="L3" t="n">
+        <v>42.4</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>33</v>
+      </c>
+      <c r="N3" t="n">
+        <v>40.6</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>32</v>
+      </c>
+      <c r="P3" t="n">
+        <v>48.4</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>91</v>
+      </c>
+      <c r="R3" t="n">
+        <v>58.1</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="T3" t="n">
+        <v>100</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
+      <c r="X3" t="n">
+        <v>50</v>
+      </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>146</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>33.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>81.2</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>66.7</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>55.1</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
@@ -1176,17 +1302,29 @@
           <t>Avg</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>75.5</v>
+      </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>53</v>
+      </c>
+      <c r="D4" t="n">
+        <v>90.2</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="F4" t="n">
+        <v>57.9</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="H4" t="n">
+        <v>63</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1194,14 +1332,23 @@
       <c r="M4" t="n">
         <v>0</v>
       </c>
+      <c r="N4" t="n">
+        <v>25</v>
+      </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="P4" t="n">
+        <v>33.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="R4" t="n">
+        <v>38.5</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -1209,20 +1356,29 @@
       <c r="W4" t="n">
         <v>0</v>
       </c>
+      <c r="X4" t="n">
+        <v>34.9</v>
+      </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
       </c>
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
+      <c r="AF4" t="n">
+        <v>42.3</v>
+      </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -1231,29 +1387,53 @@
           <t>Below Avg</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>28.6</v>
+      </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>57.1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>14.3</v>
       </c>
       <c r="G5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>20</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>20</v>
       </c>
       <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="P5" t="n">
+        <v>33.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -1264,11 +1444,17 @@
       <c r="W5" t="n">
         <v>0</v>
       </c>
+      <c r="X5" t="n">
+        <v>44.4</v>
+      </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>81.8</v>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1276,8 +1462,11 @@
       <c r="AE5" t="n">
         <v>0</v>
       </c>
+      <c r="AF5" t="n">
+        <v>55</v>
+      </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1286,29 +1475,50 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>90.90000000000001</v>
+      </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="D6" t="n">
+        <v>75</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>83.3</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
+      <c r="J6" t="n">
+        <v>50</v>
+      </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>40.7</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="N6" t="n">
+        <v>25</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="P6" t="n">
+        <v>12.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1319,20 +1529,32 @@
       <c r="W6" t="n">
         <v>0</v>
       </c>
+      <c r="X6" t="n">
+        <v>20</v>
+      </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>26.3</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>16.7</v>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
       </c>
+      <c r="AF6" t="n">
+        <v>62.5</v>
+      </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1341,62 +1563,101 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="B7" t="n">
+        <v>66.7</v>
+      </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>675</v>
+      </c>
+      <c r="D7" t="n">
+        <v>64.59999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>492</v>
+      </c>
+      <c r="F7" t="n">
+        <v>64.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>243</v>
+      </c>
+      <c r="H7" t="n">
+        <v>56.7</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>238</v>
+      </c>
+      <c r="J7" t="n">
+        <v>31.4</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>188</v>
+      </c>
+      <c r="L7" t="n">
+        <v>22.4</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>312</v>
+      </c>
+      <c r="N7" t="n">
+        <v>23.8</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>143</v>
+      </c>
+      <c r="P7" t="n">
+        <v>21.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>2430</v>
+      </c>
+      <c r="R7" t="n">
+        <v>53.3</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="T7" t="n">
+        <v>41.7</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="V7" t="n">
+        <v>53.1</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="X7" t="n">
-        <v>19.3</v>
+        <v>37.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>187</v>
+        <v>795</v>
       </c>
       <c r="Z7" t="n">
-        <v>100</v>
+        <v>57.1</v>
       </c>
       <c r="AA7" t="n">
-        <v>1</v>
+        <v>91</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>62.5</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>37.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>1</v>
+        <v>35</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>50.9</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>